<commit_message>
demographic form's age section modified
</commit_message>
<xml_diff>
--- a/demoForm.xlsx
+++ b/demoForm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPPA\CMKL\Animation_Project\Summer\Experiment_Workflows\Testing1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\psychopyexperiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC34BB6D-CD8A-46D9-92AC-1031000680ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CCDBE8-6633-4174-A0CF-22BACED3EAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1464" yWindow="1464" windowWidth="12960" windowHeight="7824" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t>index</t>
   </si>
@@ -293,9 +293,6 @@
     <t>What is your age?</t>
   </si>
   <si>
-    <t>free text</t>
-  </si>
-  <si>
     <t>What is your gender?</t>
   </si>
   <si>
@@ -318,6 +315,12 @@
   </si>
   <si>
     <t>A1 - Beginner, A2 - Elementary, B1 - Intermediate, B2 - Upper-intermediate, C1 - Advanced, C2 - Proficient</t>
+  </si>
+  <si>
+    <t>horiz</t>
+  </si>
+  <si>
+    <t>18, 19, 20, 21, 22, 23, 24, 25</t>
   </si>
 </sst>
 </file>
@@ -691,19 +694,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z5"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="12.69921875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.80859375" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" customWidth="1"/>
+    <col min="1" max="1" width="5.796875" customWidth="1"/>
+    <col min="2" max="2" width="31.09765625" customWidth="1"/>
+    <col min="3" max="3" width="13.69921875" customWidth="1"/>
     <col min="4" max="4" width="84" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="22.47265625" customWidth="1"/>
-    <col min="7" max="7" width="9.33203125" customWidth="1"/>
-    <col min="8" max="13" width="13.6640625" customWidth="1"/>
-    <col min="14" max="26" width="7.6640625" customWidth="1"/>
+    <col min="5" max="6" width="22.5" customWidth="1"/>
+    <col min="7" max="7" width="9.296875" customWidth="1"/>
+    <col min="8" max="13" width="13.69921875" customWidth="1"/>
+    <col min="14" max="26" width="7.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -757,7 +760,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -765,14 +768,24 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="3"/>
+      <c r="G2" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="H2" s="2"/>
+      <c r="I2">
+        <v>0.5</v>
+      </c>
       <c r="J2" s="2"/>
+      <c r="K2">
+        <v>1</v>
+      </c>
       <c r="O2" s="4"/>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
@@ -786,73 +799,73 @@
       <c r="Y2" s="5"/>
       <c r="Z2" s="5"/>
     </row>
-    <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
       <c r="I3">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="K3">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I4">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="K4">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I5">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="K5">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>